<commit_message>
finish export patient search
</commit_message>
<xml_diff>
--- a/Hospital/wwwroot/Template/UrologyTemplate.xlsx
+++ b/Hospital/wwwroot/Template/UrologyTemplate.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Salam\ZA\Hospital\Hospital\Hospital\wwwroot\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8398C35B-9AC7-4AF6-83A9-8FC28858FB09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2A4F162-4029-44B1-83D9-C23511B42501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Items by MPN-temp" sheetId="6" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Items by MPN-temp'!$A$4:$AS$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$4:$AS$6</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>

</xml_diff>